<commit_message>
Actualizar reglas de ajuste y ejecucion local
</commit_message>
<xml_diff>
--- a/Produccion Astroflores BL25-26-27-28 a la Semana 15.xlsx
+++ b/Produccion Astroflores BL25-26-27-28 a la Semana 15.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Astroflores" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Astroflores!$A$1:$R$559</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Astroflores!$A$1:$R$567</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
   <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2250" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2282" uniqueCount="33">
   <si>
     <t>Anio</t>
   </si>
@@ -555,7 +555,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Hoja1" filterMode="1"/>
-  <dimension ref="A1:R559"/>
+  <dimension ref="A1:R567"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.375" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="9" style="2" bestFit="1" customWidth="1"/>
@@ -906,7 +906,7 @@
         <v>1.3786031673692607</v>
       </c>
     </row>
-    <row r="7" spans="1:18">
+    <row r="7" spans="1:18" hidden="1">
       <c r="A7" s="3">
         <v>2025</v>
       </c>
@@ -1346,7 +1346,7 @@
         <v>1.2304887774866127</v>
       </c>
     </row>
-    <row r="15" spans="1:18">
+    <row r="15" spans="1:18" hidden="1">
       <c r="A15" s="3">
         <v>2025</v>
       </c>
@@ -1786,7 +1786,7 @@
         <v>2.1533553606015725</v>
       </c>
     </row>
-    <row r="23" spans="1:17">
+    <row r="23" spans="1:17" hidden="1">
       <c r="A23" s="3">
         <v>2025</v>
       </c>
@@ -2226,7 +2226,7 @@
         <v>4.3181041358095023</v>
       </c>
     </row>
-    <row r="31" spans="1:17">
+    <row r="31" spans="1:17" hidden="1">
       <c r="A31" s="3">
         <v>2025</v>
       </c>
@@ -2666,7 +2666,7 @@
         <v>6.2435912042839243</v>
       </c>
     </row>
-    <row r="39" spans="1:17">
+    <row r="39" spans="1:17" hidden="1">
       <c r="A39" s="3">
         <v>2025</v>
       </c>
@@ -3106,7 +3106,7 @@
         <v>3.3610573088754703</v>
       </c>
     </row>
-    <row r="47" spans="1:17">
+    <row r="47" spans="1:17" hidden="1">
       <c r="A47" s="3">
         <v>2025</v>
       </c>
@@ -3546,7 +3546,7 @@
         <v>2.0849948729634273</v>
       </c>
     </row>
-    <row r="55" spans="1:17">
+    <row r="55" spans="1:17" hidden="1">
       <c r="A55" s="3">
         <v>2025</v>
       </c>
@@ -3986,7 +3986,7 @@
         <v>1.2874558505184004</v>
       </c>
     </row>
-    <row r="63" spans="1:17">
+    <row r="63" spans="1:17" hidden="1">
       <c r="A63" s="3">
         <v>2025</v>
       </c>
@@ -4426,7 +4426,7 @@
         <v>1.2760624359120429</v>
       </c>
     </row>
-    <row r="71" spans="1:17">
+    <row r="71" spans="1:17" hidden="1">
       <c r="A71" s="3">
         <v>2025</v>
       </c>
@@ -4866,7 +4866,7 @@
         <v>1.3558163381565456</v>
       </c>
     </row>
-    <row r="79" spans="1:17">
+    <row r="79" spans="1:17" hidden="1">
       <c r="A79" s="3">
         <v>2025</v>
       </c>
@@ -5306,7 +5306,7 @@
         <v>1.3330295089438304</v>
       </c>
     </row>
-    <row r="87" spans="1:17">
+    <row r="87" spans="1:17" hidden="1">
       <c r="A87" s="3">
         <v>2025</v>
       </c>
@@ -5746,7 +5746,7 @@
         <v>1.15073487524211</v>
       </c>
     </row>
-    <row r="95" spans="1:17">
+    <row r="95" spans="1:17" hidden="1">
       <c r="A95" s="3">
         <v>2025</v>
       </c>
@@ -6186,7 +6186,7 @@
         <v>1.2304887774866127</v>
       </c>
     </row>
-    <row r="103" spans="1:17">
+    <row r="103" spans="1:17" hidden="1">
       <c r="A103" s="3">
         <v>2025</v>
       </c>
@@ -6626,7 +6626,7 @@
         <v>1.3899965819756182</v>
       </c>
     </row>
-    <row r="111" spans="1:17">
+    <row r="111" spans="1:17" hidden="1">
       <c r="A111" s="3">
         <v>2025</v>
       </c>
@@ -7066,7 +7066,7 @@
         <v>1.15073487524211</v>
       </c>
     </row>
-    <row r="119" spans="1:17">
+    <row r="119" spans="1:17" hidden="1">
       <c r="A119" s="3">
         <v>2025</v>
       </c>
@@ -7506,7 +7506,7 @@
         <v>1.7431924347727015</v>
       </c>
     </row>
-    <row r="127" spans="1:17">
+    <row r="127" spans="1:17" hidden="1">
       <c r="A127" s="3">
         <v>2025</v>
       </c>
@@ -7946,7 +7946,7 @@
         <v>3.6117124302153356</v>
       </c>
     </row>
-    <row r="135" spans="1:17">
+    <row r="135" spans="1:17" hidden="1">
       <c r="A135" s="3">
         <v>2025</v>
       </c>
@@ -8386,7 +8386,7 @@
         <v>4.8080209638828757</v>
       </c>
     </row>
-    <row r="143" spans="1:17">
+    <row r="143" spans="1:17" hidden="1">
       <c r="A143" s="3">
         <v>2025</v>
       </c>
@@ -8826,7 +8826,7 @@
         <v>2.0736014583570697</v>
       </c>
     </row>
-    <row r="151" spans="1:17">
+    <row r="151" spans="1:17" hidden="1">
       <c r="A151" s="3">
         <v>2025</v>
       </c>
@@ -9266,7 +9266,7 @@
         <v>2.1989290190270023</v>
       </c>
     </row>
-    <row r="159" spans="1:17">
+    <row r="159" spans="1:17" hidden="1">
       <c r="A159" s="3">
         <v>2025</v>
       </c>
@@ -9706,7 +9706,7 @@
         <v>1.6064714594964111</v>
       </c>
     </row>
-    <row r="167" spans="1:17">
+    <row r="167" spans="1:17" hidden="1">
       <c r="A167" s="3">
         <v>2025</v>
       </c>
@@ -10146,7 +10146,7 @@
         <v>1.4127834111883333</v>
       </c>
     </row>
-    <row r="175" spans="1:17">
+    <row r="175" spans="1:17" hidden="1">
       <c r="A175" s="3">
         <v>2025</v>
       </c>
@@ -10586,7 +10586,7 @@
         <v>1.2988492651247578</v>
       </c>
     </row>
-    <row r="183" spans="1:17">
+    <row r="183" spans="1:17" hidden="1">
       <c r="A183" s="3">
         <v>2025</v>
       </c>
@@ -11026,7 +11026,7 @@
         <v>0.91147316850860205</v>
       </c>
     </row>
-    <row r="191" spans="1:17">
+    <row r="191" spans="1:17" hidden="1">
       <c r="A191" s="3">
         <v>2025</v>
       </c>
@@ -11466,7 +11466,7 @@
         <v>0.92286658311495962</v>
       </c>
     </row>
-    <row r="199" spans="1:17">
+    <row r="199" spans="1:17" hidden="1">
       <c r="A199" s="3">
         <v>2025</v>
       </c>
@@ -11906,7 +11906,7 @@
         <v>0.85450609547681444</v>
       </c>
     </row>
-    <row r="207" spans="1:17">
+    <row r="207" spans="1:17" hidden="1">
       <c r="A207" s="3">
         <v>2025</v>
       </c>
@@ -12346,7 +12346,7 @@
         <v>0.70639170559416664</v>
       </c>
     </row>
-    <row r="215" spans="1:17">
+    <row r="215" spans="1:17" hidden="1">
       <c r="A215" s="3">
         <v>2025</v>
       </c>
@@ -12786,7 +12786,7 @@
         <v>0.92286658311495962</v>
       </c>
     </row>
-    <row r="223" spans="1:17">
+    <row r="223" spans="1:17" hidden="1">
       <c r="A223" s="3">
         <v>2025</v>
       </c>
@@ -13226,7 +13226,7 @@
         <v>0.99122707075310479</v>
       </c>
     </row>
-    <row r="231" spans="1:17">
+    <row r="231" spans="1:17" hidden="1">
       <c r="A231" s="3">
         <v>2025</v>
       </c>
@@ -13666,7 +13666,7 @@
         <v>1.5950780448900537</v>
       </c>
     </row>
-    <row r="239" spans="1:17">
+    <row r="239" spans="1:17" hidden="1">
       <c r="A239" s="3">
         <v>2025</v>
       </c>
@@ -14106,7 +14106,7 @@
         <v>2.8255668223766666</v>
       </c>
     </row>
-    <row r="247" spans="1:17">
+    <row r="247" spans="1:17" hidden="1">
       <c r="A247" s="3">
         <v>2025</v>
       </c>
@@ -14546,7 +14546,7 @@
         <v>1.7773726785917741</v>
       </c>
     </row>
-    <row r="255" spans="1:17">
+    <row r="255" spans="1:17" hidden="1">
       <c r="A255" s="3">
         <v>2025</v>
       </c>
@@ -14986,7 +14986,7 @@
         <v>1.4811438988264785</v>
       </c>
     </row>
-    <row r="263" spans="1:17">
+    <row r="263" spans="1:17" hidden="1">
       <c r="A263" s="3">
         <v>2025</v>
       </c>
@@ -15426,7 +15426,7 @@
         <v>1.8343397516235616</v>
       </c>
     </row>
-    <row r="271" spans="1:17">
+    <row r="271" spans="1:17" hidden="1">
       <c r="A271" s="3">
         <v>2025</v>
       </c>
@@ -15866,7 +15866,7 @@
         <v>2.1077817021761422</v>
       </c>
     </row>
-    <row r="279" spans="1:17">
+    <row r="279" spans="1:17" hidden="1">
       <c r="A279" s="3">
         <v>2025</v>
       </c>
@@ -16306,7 +16306,7 @@
         <v>1.538110971858266</v>
       </c>
     </row>
-    <row r="287" spans="1:17">
+    <row r="287" spans="1:17" hidden="1">
       <c r="A287" s="3">
         <v>2025</v>
       </c>
@@ -16746,7 +16746,7 @@
         <v>1.3558163381565456</v>
       </c>
     </row>
-    <row r="295" spans="1:17">
+    <row r="295" spans="1:17" hidden="1">
       <c r="A295" s="3">
         <v>2025</v>
       </c>
@@ -17186,7 +17186,7 @@
         <v>1.5950780448900537</v>
       </c>
     </row>
-    <row r="303" spans="1:17">
+    <row r="303" spans="1:17" hidden="1">
       <c r="A303" s="3">
         <v>2025</v>
       </c>
@@ -17626,7 +17626,7 @@
         <v>2.2672895066651475</v>
       </c>
     </row>
-    <row r="311" spans="1:17">
+    <row r="311" spans="1:17" hidden="1">
       <c r="A311" s="3">
         <v>2025</v>
       </c>
@@ -18066,7 +18066,7 @@
         <v>2.0052409707189245</v>
       </c>
     </row>
-    <row r="319" spans="1:17">
+    <row r="319" spans="1:17" hidden="1">
       <c r="A319" s="3">
         <v>2025</v>
       </c>
@@ -18506,7 +18506,7 @@
         <v>1.3444229235501881</v>
       </c>
     </row>
-    <row r="327" spans="1:17">
+    <row r="327" spans="1:17" hidden="1">
       <c r="A327" s="3">
         <v>2025</v>
       </c>
@@ -18946,7 +18946,7 @@
         <v>0.91147316850860205</v>
       </c>
     </row>
-    <row r="335" spans="1:17">
+    <row r="335" spans="1:17" hidden="1">
       <c r="A335" s="3">
         <v>2025</v>
       </c>
@@ -19386,7 +19386,7 @@
         <v>0.99122707075310479</v>
       </c>
     </row>
-    <row r="343" spans="1:17">
+    <row r="343" spans="1:17" hidden="1">
       <c r="A343" s="3">
         <v>2025</v>
       </c>
@@ -19826,7 +19826,7 @@
         <v>1.4925373134328359</v>
       </c>
     </row>
-    <row r="351" spans="1:17">
+    <row r="351" spans="1:17" hidden="1">
       <c r="A351" s="3">
         <v>2025</v>
       </c>
@@ -20266,7 +20266,7 @@
         <v>1.6862253617409138</v>
       </c>
     </row>
-    <row r="359" spans="1:17">
+    <row r="359" spans="1:17" hidden="1">
       <c r="A359" s="3">
         <v>2025</v>
       </c>
@@ -20706,7 +20706,7 @@
         <v>1.6520451179218412</v>
       </c>
     </row>
-    <row r="367" spans="1:17">
+    <row r="367" spans="1:17" hidden="1">
       <c r="A367" s="3">
         <v>2025</v>
       </c>
@@ -21146,7 +21146,7 @@
         <v>1.9027002392617067</v>
       </c>
     </row>
-    <row r="375" spans="1:17">
+    <row r="375" spans="1:17" hidden="1">
       <c r="A375" s="3">
         <v>2025</v>
       </c>
@@ -21586,7 +21586,7 @@
         <v>1.6406517033154837</v>
       </c>
     </row>
-    <row r="383" spans="1:17">
+    <row r="383" spans="1:17" hidden="1">
       <c r="A383" s="3">
         <v>2025</v>
       </c>
@@ -22026,7 +22026,7 @@
         <v>1.5039307280391934</v>
       </c>
     </row>
-    <row r="391" spans="1:17">
+    <row r="391" spans="1:17" hidden="1">
       <c r="A391" s="3">
         <v>2025</v>
       </c>
@@ -22466,7 +22466,7 @@
         <v>1.8685199954426341</v>
       </c>
     </row>
-    <row r="399" spans="1:17">
+    <row r="399" spans="1:17" hidden="1">
       <c r="A399" s="3">
         <v>2025</v>
       </c>
@@ -22906,7 +22906,7 @@
         <v>1.9027002392617067</v>
       </c>
     </row>
-    <row r="407" spans="1:17">
+    <row r="407" spans="1:17" hidden="1">
       <c r="A407" s="3">
         <v>2025</v>
       </c>
@@ -23346,7 +23346,7 @@
         <v>2.1305685313888572</v>
       </c>
     </row>
-    <row r="415" spans="1:17">
+    <row r="415" spans="1:17" hidden="1">
       <c r="A415" s="3">
         <v>2025</v>
       </c>
@@ -23786,7 +23786,7 @@
         <v>1.8799134100489918</v>
       </c>
     </row>
-    <row r="423" spans="1:17">
+    <row r="423" spans="1:17" hidden="1">
       <c r="A423" s="3">
         <v>2026</v>
       </c>
@@ -24226,7 +24226,7 @@
         <v>1.9368804830807793</v>
       </c>
     </row>
-    <row r="431" spans="1:17">
+    <row r="431" spans="1:17" hidden="1">
       <c r="A431" s="3">
         <v>2026</v>
       </c>
@@ -24666,7 +24666,7 @@
         <v>1.4013899965819756</v>
       </c>
     </row>
-    <row r="439" spans="1:17">
+    <row r="439" spans="1:17" hidden="1">
       <c r="A439" s="3">
         <v>2026</v>
       </c>
@@ -25106,7 +25106,7 @@
         <v>3.3496638942691126</v>
       </c>
     </row>
-    <row r="447" spans="1:17">
+    <row r="447" spans="1:17" hidden="1">
       <c r="A447" s="3">
         <v>2026</v>
       </c>
@@ -25546,7 +25546,7 @@
         <v>5.8448216930614105</v>
       </c>
     </row>
-    <row r="455" spans="1:17">
+    <row r="455" spans="1:17" hidden="1">
       <c r="A455" s="3">
         <v>2026</v>
       </c>
@@ -25986,7 +25986,7 @@
         <v>2.7002392617067335</v>
       </c>
     </row>
-    <row r="463" spans="1:17">
+    <row r="463" spans="1:17" hidden="1">
       <c r="A463" s="3">
         <v>2026</v>
       </c>
@@ -26426,7 +26426,7 @@
         <v>2.6546656032813036</v>
       </c>
     </row>
-    <row r="471" spans="1:17">
+    <row r="471" spans="1:17" hidden="1">
       <c r="A471" s="3">
         <v>2026</v>
       </c>
@@ -26866,7 +26866,7 @@
         <v>2.1419619459952148</v>
       </c>
     </row>
-    <row r="479" spans="1:17">
+    <row r="479" spans="1:17" hidden="1">
       <c r="A479" s="3">
         <v>2026</v>
       </c>
@@ -27306,7 +27306,7 @@
         <v>1.0368007291785348</v>
       </c>
     </row>
-    <row r="487" spans="1:17">
+    <row r="487" spans="1:17" hidden="1">
       <c r="A487" s="3">
         <v>2026</v>
       </c>
@@ -27746,7 +27746,7 @@
         <v>2.3926170673350806</v>
       </c>
     </row>
-    <row r="495" spans="1:17">
+    <row r="495" spans="1:17" hidden="1">
       <c r="A495" s="3">
         <v>2026</v>
       </c>
@@ -28186,7 +28186,7 @@
         <v>1.8913068246553493</v>
       </c>
     </row>
-    <row r="503" spans="1:17">
+    <row r="503" spans="1:17" hidden="1">
       <c r="A503" s="3">
         <v>2026</v>
       </c>
@@ -28626,7 +28626,7 @@
         <v>1.4127834111883333</v>
       </c>
     </row>
-    <row r="511" spans="1:17">
+    <row r="511" spans="1:17" hidden="1">
       <c r="A511" s="3">
         <v>2026</v>
       </c>
@@ -28866,7 +28866,7 @@
         <v>20</v>
       </c>
       <c r="G515" s="3" t="str">
-        <f t="shared" ref="G515:G559" si="16">+E515&amp;F515</f>
+        <f t="shared" ref="G515:G567" si="16">+E515&amp;F515</f>
         <v>025PINK MONDIAL</v>
       </c>
       <c r="H515" s="6">
@@ -28897,7 +28897,7 @@
         <v>13.861755952380944</v>
       </c>
       <c r="Q515" s="8">
-        <f t="shared" ref="Q515:Q559" si="17">+H515/K515</f>
+        <f t="shared" ref="Q515:Q567" si="17">+H515/K515</f>
         <v>1.8148078514202977</v>
       </c>
     </row>
@@ -29066,7 +29066,7 @@
         <v>2.4951577987922979</v>
       </c>
     </row>
-    <row r="519" spans="1:17">
+    <row r="519" spans="1:17" hidden="1">
       <c r="A519" s="3">
         <v>2026</v>
       </c>
@@ -29451,7 +29451,7 @@
         <v>1.8343397516235616</v>
       </c>
     </row>
-    <row r="526" spans="1:17">
+    <row r="526" spans="1:17" hidden="1">
       <c r="A526" s="3">
         <v>2026</v>
       </c>
@@ -29616,7 +29616,7 @@
         <v>2.4820115511695779</v>
       </c>
     </row>
-    <row r="529" spans="1:17" hidden="1">
+    <row r="529" spans="1:18" hidden="1">
       <c r="A529" s="3">
         <v>2026</v>
       </c>
@@ -29671,7 +29671,7 @@
         <v>2.1240576198237564</v>
       </c>
     </row>
-    <row r="530" spans="1:17" hidden="1">
+    <row r="530" spans="1:18" hidden="1">
       <c r="A530" s="3">
         <v>2026</v>
       </c>
@@ -29726,7 +29726,7 @@
         <v>3.3479110612527498</v>
       </c>
     </row>
-    <row r="531" spans="1:17" hidden="1">
+    <row r="531" spans="1:18" hidden="1">
       <c r="A531" s="3">
         <v>2026</v>
       </c>
@@ -29781,7 +29781,7 @@
         <v>4.0928650932068953</v>
       </c>
     </row>
-    <row r="532" spans="1:17" hidden="1">
+    <row r="532" spans="1:18" hidden="1">
       <c r="A532" s="3">
         <v>2026</v>
       </c>
@@ -29836,7 +29836,7 @@
         <v>2.472370969579583</v>
       </c>
     </row>
-    <row r="533" spans="1:17">
+    <row r="533" spans="1:18" hidden="1">
       <c r="A533" s="3">
         <v>2026</v>
       </c>
@@ -29891,7 +29891,7 @@
         <v>2.1305685313888572</v>
       </c>
     </row>
-    <row r="534" spans="1:17" hidden="1">
+    <row r="534" spans="1:18" hidden="1">
       <c r="A534" s="3">
         <v>2026</v>
       </c>
@@ -29946,7 +29946,7 @@
         <v>2.2296035968133494</v>
       </c>
     </row>
-    <row r="535" spans="1:17" hidden="1">
+    <row r="535" spans="1:18" hidden="1">
       <c r="A535" s="3">
         <v>2026</v>
       </c>
@@ -30001,7 +30001,7 @@
         <v>4.091112260190533</v>
       </c>
     </row>
-    <row r="536" spans="1:17" hidden="1">
+    <row r="536" spans="1:18" hidden="1">
       <c r="A536" s="3">
         <v>2026</v>
       </c>
@@ -30056,7 +30056,7 @@
         <v>0.56967073031787618</v>
       </c>
     </row>
-    <row r="537" spans="1:17" hidden="1">
+    <row r="537" spans="1:18" hidden="1">
       <c r="A537" s="3">
         <v>2026</v>
       </c>
@@ -30110,8 +30110,11 @@
         <f t="shared" si="17"/>
         <v>1.7171500298192053</v>
       </c>
-    </row>
-    <row r="538" spans="1:17" hidden="1">
+      <c r="R537" s="2">
+        <v>6217</v>
+      </c>
+    </row>
+    <row r="538" spans="1:18" hidden="1">
       <c r="A538" s="3">
         <v>2026</v>
       </c>
@@ -30165,8 +30168,11 @@
         <f t="shared" si="17"/>
         <v>8.3126352967984509</v>
       </c>
-    </row>
-    <row r="539" spans="1:17" hidden="1">
+      <c r="R538" s="2">
+        <v>11646</v>
+      </c>
+    </row>
+    <row r="539" spans="1:18" hidden="1">
       <c r="A539" s="3">
         <v>2026</v>
       </c>
@@ -30220,8 +30226,11 @@
         <f t="shared" si="17"/>
         <v>2.41189823051507</v>
       </c>
-    </row>
-    <row r="540" spans="1:17" hidden="1">
+      <c r="R539" s="2">
+        <v>8016</v>
+      </c>
+    </row>
+    <row r="540" spans="1:18" hidden="1">
       <c r="A540" s="3">
         <v>2026</v>
       </c>
@@ -30275,8 +30284,11 @@
         <f t="shared" si="17"/>
         <v>1.7431924347727015</v>
       </c>
-    </row>
-    <row r="541" spans="1:17">
+      <c r="R540" s="2">
+        <v>5985</v>
+      </c>
+    </row>
+    <row r="541" spans="1:18" hidden="1">
       <c r="A541" s="3">
         <v>2026</v>
       </c>
@@ -30330,8 +30342,11 @@
         <f t="shared" si="17"/>
         <v>1.7204056055599863</v>
       </c>
-    </row>
-    <row r="542" spans="1:17" hidden="1">
+      <c r="R541" s="2">
+        <v>5799</v>
+      </c>
+    </row>
+    <row r="542" spans="1:18" hidden="1">
       <c r="A542" s="3">
         <v>2026</v>
       </c>
@@ -30385,8 +30400,11 @@
         <f t="shared" si="17"/>
         <v>1.6827196957081882</v>
       </c>
-    </row>
-    <row r="543" spans="1:17" hidden="1">
+      <c r="R542" s="2">
+        <v>6641</v>
+      </c>
+    </row>
+    <row r="543" spans="1:18">
       <c r="A543" s="3">
         <v>2026</v>
       </c>
@@ -30440,8 +30458,11 @@
         <f t="shared" si="17"/>
         <v>3.7861193153434236</v>
       </c>
-    </row>
-    <row r="544" spans="1:17" hidden="1">
+      <c r="R543" s="2">
+        <v>14933</v>
+      </c>
+    </row>
+    <row r="544" spans="1:18" hidden="1">
       <c r="A544" s="3">
         <v>2026</v>
       </c>
@@ -30496,7 +30517,7 @@
         <v>0.8658995100831719</v>
       </c>
     </row>
-    <row r="545" spans="1:17" hidden="1">
+    <row r="545" spans="1:18" hidden="1">
       <c r="A545" s="3">
         <v>2026</v>
       </c>
@@ -30550,8 +30571,11 @@
         <f t="shared" si="17"/>
         <v>3.4587145150386838</v>
       </c>
-    </row>
-    <row r="546" spans="1:17" hidden="1">
+      <c r="R545" s="2">
+        <v>12165</v>
+      </c>
+    </row>
+    <row r="546" spans="1:18" hidden="1">
       <c r="A546" s="3">
         <v>2026</v>
       </c>
@@ -30605,8 +30629,11 @@
         <f t="shared" si="17"/>
         <v>8.5496183206106871</v>
       </c>
-    </row>
-    <row r="547" spans="1:17" hidden="1">
+      <c r="R546" s="2">
+        <v>12252</v>
+      </c>
+    </row>
+    <row r="547" spans="1:18" hidden="1">
       <c r="A547" s="3">
         <v>2026</v>
       </c>
@@ -30660,8 +30687,11 @@
         <f t="shared" si="17"/>
         <v>3.8772666321942837</v>
       </c>
-    </row>
-    <row r="548" spans="1:17" hidden="1">
+      <c r="R547" s="2">
+        <v>13928</v>
+      </c>
+    </row>
+    <row r="548" spans="1:18" hidden="1">
       <c r="A548" s="3">
         <v>2026</v>
       </c>
@@ -30715,8 +30745,11 @@
         <f t="shared" si="17"/>
         <v>3.6117124302153356</v>
       </c>
-    </row>
-    <row r="549" spans="1:17">
+      <c r="R548" s="2">
+        <v>13719</v>
+      </c>
+    </row>
+    <row r="549" spans="1:18" hidden="1">
       <c r="A549" s="3">
         <v>2026</v>
       </c>
@@ -30770,8 +30803,11 @@
         <f t="shared" si="17"/>
         <v>3.4863848695454029</v>
       </c>
-    </row>
-    <row r="550" spans="1:17" hidden="1">
+      <c r="R549" s="2">
+        <v>12377</v>
+      </c>
+    </row>
+    <row r="550" spans="1:18" hidden="1">
       <c r="A550" s="3">
         <v>2026</v>
       </c>
@@ -30825,8 +30861,11 @@
         <f t="shared" si="17"/>
         <v>1.2830737679774935</v>
       </c>
-    </row>
-    <row r="551" spans="1:17" hidden="1">
+      <c r="R550" s="2">
+        <v>4876</v>
+      </c>
+    </row>
+    <row r="551" spans="1:18">
       <c r="A551" s="3">
         <v>2026</v>
       </c>
@@ -30880,8 +30919,11 @@
         <f t="shared" si="17"/>
         <v>7.5406876363923185</v>
       </c>
-    </row>
-    <row r="552" spans="1:17" hidden="1">
+      <c r="R551" s="2">
+        <v>29385</v>
+      </c>
+    </row>
+    <row r="552" spans="1:18" hidden="1">
       <c r="A552" s="3">
         <v>2026</v>
       </c>
@@ -30936,7 +30978,7 @@
         <v>0.91716987581178078</v>
       </c>
     </row>
-    <row r="553" spans="1:17" hidden="1">
+    <row r="553" spans="1:18" hidden="1">
       <c r="A553" s="3">
         <v>2026</v>
       </c>
@@ -30990,8 +31032,11 @@
         <f t="shared" si="17"/>
         <v>2.9785635588333137</v>
       </c>
-    </row>
-    <row r="554" spans="1:17" hidden="1">
+      <c r="R553" s="2">
+        <v>10796</v>
+      </c>
+    </row>
+    <row r="554" spans="1:18" hidden="1">
       <c r="A554" s="3">
         <v>2026</v>
       </c>
@@ -31045,8 +31090,11 @@
         <f t="shared" si="17"/>
         <v>6.5990657400022785</v>
       </c>
-    </row>
-    <row r="555" spans="1:17" hidden="1">
+      <c r="R554" s="2">
+        <v>10080</v>
+      </c>
+    </row>
+    <row r="555" spans="1:18" hidden="1">
       <c r="A555" s="3">
         <v>2026</v>
       </c>
@@ -31100,8 +31148,11 @@
         <f t="shared" si="17"/>
         <v>3.4916433685944908</v>
       </c>
-    </row>
-    <row r="556" spans="1:17" hidden="1">
+      <c r="R555" s="2">
+        <v>12228</v>
+      </c>
+    </row>
+    <row r="556" spans="1:18" hidden="1">
       <c r="A556" s="3">
         <v>2026</v>
       </c>
@@ -31155,8 +31206,11 @@
         <f t="shared" si="17"/>
         <v>4.8080209638828757</v>
       </c>
-    </row>
-    <row r="557" spans="1:17">
+      <c r="R556" s="2">
+        <v>16946</v>
+      </c>
+    </row>
+    <row r="557" spans="1:18" hidden="1">
       <c r="A557" s="3">
         <v>2026</v>
       </c>
@@ -31210,8 +31264,11 @@
         <f t="shared" si="17"/>
         <v>4.5687592571493676</v>
       </c>
-    </row>
-    <row r="558" spans="1:17" hidden="1">
+      <c r="R557" s="2">
+        <v>15072</v>
+      </c>
+    </row>
+    <row r="558" spans="1:18" hidden="1">
       <c r="A558" s="3">
         <v>2026</v>
       </c>
@@ -31265,8 +31322,11 @@
         <f t="shared" si="17"/>
         <v>2.6292495245440444</v>
       </c>
-    </row>
-    <row r="559" spans="1:17" hidden="1">
+      <c r="R558" s="2">
+        <v>9010</v>
+      </c>
+    </row>
+    <row r="559" spans="1:18">
       <c r="A559" s="3">
         <v>2026</v>
       </c>
@@ -31320,13 +31380,490 @@
         <f t="shared" si="17"/>
         <v>6.6151918037528157</v>
       </c>
+      <c r="R559" s="2">
+        <v>26535</v>
+      </c>
+    </row>
+    <row r="560" spans="1:18" hidden="1">
+      <c r="A560" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B560" s="3">
+        <v>19</v>
+      </c>
+      <c r="C560" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D560" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E560" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F560" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G560" s="3" t="str">
+        <f t="shared" si="16"/>
+        <v>026PURPLE BUBBLY</v>
+      </c>
+      <c r="H560" s="3">
+        <v>670</v>
+      </c>
+      <c r="I560" s="3">
+        <v>1331</v>
+      </c>
+      <c r="J560" s="3">
+        <v>1232</v>
+      </c>
+      <c r="K560" s="3">
+        <v>1755.4</v>
+      </c>
+      <c r="L560" s="3">
+        <v>12800</v>
+      </c>
+      <c r="M560" s="3">
+        <v>12</v>
+      </c>
+      <c r="N560" s="3">
+        <v>13.801155115511554</v>
+      </c>
+      <c r="O560" s="3">
+        <v>14.032838283828401</v>
+      </c>
+      <c r="P560" s="3">
+        <v>13.571947194719476</v>
+      </c>
+      <c r="Q560" s="8">
+        <f t="shared" si="17"/>
+        <v>0.38167938931297707</v>
+      </c>
+    </row>
+    <row r="561" spans="1:18" hidden="1">
+      <c r="A561" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B561" s="3">
+        <v>19</v>
+      </c>
+      <c r="C561" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D561" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E561" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F561" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G561" s="3" t="str">
+        <f t="shared" si="16"/>
+        <v>025PINK MONDIAL</v>
+      </c>
+      <c r="H561" s="3">
+        <v>5800</v>
+      </c>
+      <c r="I561" s="3">
+        <v>6637</v>
+      </c>
+      <c r="J561" s="3">
+        <v>6034</v>
+      </c>
+      <c r="K561" s="3">
+        <v>3071.9505625000002</v>
+      </c>
+      <c r="L561" s="3">
+        <v>22400</v>
+      </c>
+      <c r="M561" s="3">
+        <v>12</v>
+      </c>
+      <c r="N561" s="3">
+        <v>13.801155115511554</v>
+      </c>
+      <c r="O561" s="3">
+        <v>14.032838283828401</v>
+      </c>
+      <c r="P561" s="3">
+        <v>13.571947194719476</v>
+      </c>
+      <c r="Q561" s="8">
+        <f t="shared" si="17"/>
+        <v>1.8880512176211168</v>
+      </c>
+      <c r="R561" s="2">
+        <v>6140</v>
+      </c>
+    </row>
+    <row r="562" spans="1:18" hidden="1">
+      <c r="A562" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B562" s="3">
+        <v>19</v>
+      </c>
+      <c r="C562" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D562" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E562" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F562" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G562" s="3" t="str">
+        <f t="shared" si="16"/>
+        <v>026LOLA</v>
+      </c>
+      <c r="H562" s="3">
+        <v>3760</v>
+      </c>
+      <c r="I562" s="3">
+        <v>5337</v>
+      </c>
+      <c r="J562" s="3">
+        <v>4852</v>
+      </c>
+      <c r="K562" s="3">
+        <v>1097.125</v>
+      </c>
+      <c r="L562" s="3">
+        <v>8000</v>
+      </c>
+      <c r="M562" s="3">
+        <v>12</v>
+      </c>
+      <c r="N562" s="3">
+        <v>13.801155115511554</v>
+      </c>
+      <c r="O562" s="3">
+        <v>14.032838283828401</v>
+      </c>
+      <c r="P562" s="3">
+        <v>13.571947194719476</v>
+      </c>
+      <c r="Q562" s="8">
+        <f t="shared" si="17"/>
+        <v>3.4271391135923435</v>
+      </c>
+      <c r="R562" s="2">
+        <v>6332</v>
+      </c>
+    </row>
+    <row r="563" spans="1:18" hidden="1">
+      <c r="A563" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B563" s="3">
+        <v>19</v>
+      </c>
+      <c r="C563" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D563" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E563" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F563" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G563" s="3" t="str">
+        <f t="shared" si="16"/>
+        <v>026PALOMA</v>
+      </c>
+      <c r="H563" s="3">
+        <v>5300</v>
+      </c>
+      <c r="I563" s="3">
+        <v>6201</v>
+      </c>
+      <c r="J563" s="3">
+        <v>5637</v>
+      </c>
+      <c r="K563" s="3">
+        <v>2852.5250000000001</v>
+      </c>
+      <c r="L563" s="3">
+        <v>20800</v>
+      </c>
+      <c r="M563" s="3">
+        <v>12</v>
+      </c>
+      <c r="N563" s="3">
+        <v>13.801155115511554</v>
+      </c>
+      <c r="O563" s="3">
+        <v>14.032838283828401</v>
+      </c>
+      <c r="P563" s="3">
+        <v>13.571947194719476</v>
+      </c>
+      <c r="Q563" s="8">
+        <f t="shared" si="17"/>
+        <v>1.8580029973444578</v>
+      </c>
+      <c r="R563" s="2">
+        <v>7250</v>
+      </c>
+    </row>
+    <row r="564" spans="1:18" hidden="1">
+      <c r="A564" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B564" s="3">
+        <v>19</v>
+      </c>
+      <c r="C564" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D564" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E564" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F564" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G564" s="3" t="str">
+        <f t="shared" si="16"/>
+        <v>027SATISFACTION</v>
+      </c>
+      <c r="H564" s="3">
+        <v>5460</v>
+      </c>
+      <c r="I564" s="3">
+        <v>7533</v>
+      </c>
+      <c r="J564" s="3">
+        <v>6848</v>
+      </c>
+      <c r="K564" s="3">
+        <v>2633.1</v>
+      </c>
+      <c r="L564" s="3">
+        <v>19200</v>
+      </c>
+      <c r="M564" s="3">
+        <v>12</v>
+      </c>
+      <c r="N564" s="3">
+        <v>13.801155115511554</v>
+      </c>
+      <c r="O564" s="3">
+        <v>14.032838283828401</v>
+      </c>
+      <c r="P564" s="3">
+        <v>13.571947194719476</v>
+      </c>
+      <c r="Q564" s="8">
+        <f t="shared" si="17"/>
+        <v>2.0736014583570697</v>
+      </c>
+      <c r="R564" s="2">
+        <v>6791</v>
+      </c>
+    </row>
+    <row r="565" spans="1:18" hidden="1">
+      <c r="A565" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B565" s="3">
+        <v>19</v>
+      </c>
+      <c r="C565" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D565" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E565" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F565" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G565" s="3" t="str">
+        <f t="shared" si="16"/>
+        <v>027TIFFANY!</v>
+      </c>
+      <c r="H565" s="3">
+        <v>5700</v>
+      </c>
+      <c r="I565" s="3">
+        <v>7461</v>
+      </c>
+      <c r="J565" s="3">
+        <v>6783</v>
+      </c>
+      <c r="K565" s="3">
+        <v>2633.1</v>
+      </c>
+      <c r="L565" s="3">
+        <v>19200</v>
+      </c>
+      <c r="M565" s="3">
+        <v>12</v>
+      </c>
+      <c r="N565" s="3">
+        <v>13.801155115511554</v>
+      </c>
+      <c r="O565" s="3">
+        <v>14.032838283828401</v>
+      </c>
+      <c r="P565" s="3">
+        <v>13.571947194719476</v>
+      </c>
+      <c r="Q565" s="8">
+        <f t="shared" si="17"/>
+        <v>2.1647487752079297</v>
+      </c>
+      <c r="R565" s="2">
+        <v>6322</v>
+      </c>
+    </row>
+    <row r="566" spans="1:18" hidden="1">
+      <c r="A566" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B566" s="3">
+        <v>19</v>
+      </c>
+      <c r="C566" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D566" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E566" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F566" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G566" s="3" t="str">
+        <f t="shared" si="16"/>
+        <v>028COTOPAXI</v>
+      </c>
+      <c r="H566" s="3">
+        <v>9540</v>
+      </c>
+      <c r="I566" s="3">
+        <v>7476</v>
+      </c>
+      <c r="J566" s="3">
+        <v>6796</v>
+      </c>
+      <c r="K566" s="3">
+        <v>2852.5250000000001</v>
+      </c>
+      <c r="L566" s="3">
+        <v>20800</v>
+      </c>
+      <c r="M566" s="3">
+        <v>14</v>
+      </c>
+      <c r="N566" s="3">
+        <v>13.801155115511554</v>
+      </c>
+      <c r="O566" s="3">
+        <v>14.032838283828401</v>
+      </c>
+      <c r="P566" s="3">
+        <v>13.571947194719476</v>
+      </c>
+      <c r="Q566" s="8">
+        <f t="shared" si="17"/>
+        <v>3.3444053952200243</v>
+      </c>
+      <c r="R566" s="2">
+        <v>8739</v>
+      </c>
+    </row>
+    <row r="567" spans="1:18">
+      <c r="A567" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B567" s="3">
+        <v>19</v>
+      </c>
+      <c r="C567" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D567" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E567" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F567" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G567" s="3" t="str">
+        <f t="shared" si="16"/>
+        <v>028DEEP PURPLE</v>
+      </c>
+      <c r="H567" s="3">
+        <v>11490</v>
+      </c>
+      <c r="I567" s="3">
+        <v>11537</v>
+      </c>
+      <c r="J567" s="3">
+        <v>10488</v>
+      </c>
+      <c r="K567" s="3">
+        <v>2852.5250000000001</v>
+      </c>
+      <c r="L567" s="3">
+        <v>20800</v>
+      </c>
+      <c r="M567" s="3">
+        <v>12</v>
+      </c>
+      <c r="N567" s="3">
+        <v>13.801155115511554</v>
+      </c>
+      <c r="O567" s="3">
+        <v>14.032838283828401</v>
+      </c>
+      <c r="P567" s="3">
+        <v>13.571947194719476</v>
+      </c>
+      <c r="Q567" s="8">
+        <f t="shared" si="17"/>
+        <v>4.0280102716014756</v>
+      </c>
+      <c r="R567" s="2">
+        <v>12785</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R559">
-    <filterColumn colId="5">
+  <autoFilter ref="A1:R567">
+    <filterColumn colId="0">
       <filters>
-        <filter val="TIFFANY"/>
-        <filter val="TIFFANY!"/>
+        <filter val="2.026"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="1">
+      <filters>
+        <filter val="16"/>
+        <filter val="17"/>
+        <filter val="18"/>
+        <filter val="19"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="5"/>
+    <filterColumn colId="6">
+      <filters>
+        <filter val="028DEEP PURPLE"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>